<commit_message>
Sync Oktoberfest schedule and program updates
</commit_message>
<xml_diff>
--- a/dist/График_подготовки_Октоберфест.xlsx
+++ b/dist/График_подготовки_Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98AA707B-6FEE-4F98-8373-5C4E2AA5C37B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E80BC18-2B88-4BE9-83CC-A275C34F2346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="69">
   <si>
     <t>График подготовки к фестивалю Октоберфест</t>
   </si>
@@ -165,9 +165,6 @@
     <t>выполнено</t>
   </si>
   <si>
-    <t>выполнено частично</t>
-  </si>
-  <si>
     <t>выполнено 28.09.26</t>
   </si>
   <si>
@@ -177,9 +174,6 @@
     <t>реклама стартовала</t>
   </si>
   <si>
-    <t>закуплено. Выполнено</t>
-  </si>
-  <si>
     <t>8.1.</t>
   </si>
   <si>
@@ -226,6 +220,33 @@
   </si>
   <si>
     <t>10.12.</t>
+  </si>
+  <si>
+    <t>выполнено частично. Получены замечания к Бюджету</t>
+  </si>
+  <si>
+    <t>4.1.</t>
+  </si>
+  <si>
+    <t>4.2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Подготовить 900 многоразовых купонов за участие в интерактивных программах победителям:
+-1 место – купон на подарочную колбаску или бокал пива + билет «Сезон»
+-2 место – купон на скидку 50% на любое одно блюдо в чеке + билет «Стандарт»
+-3 место – купон на скидку 30% на любое одно блюдо в чеке+ билет «Стандарт»
+</t>
+  </si>
+  <si>
+    <t>Подготовить 27 подарочных билетов за участие в интерактивных программах победителям:
+Билет «Сезон» - 9 шт
+Билет «Стандарт» - 18 шт</t>
+  </si>
+  <si>
+    <t>19.10.26.</t>
+  </si>
+  <si>
+    <t>Выполнено</t>
   </si>
 </sst>
 </file>
@@ -652,11 +673,11 @@
     <tabColor rgb="FF1F4E78"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:E40"/>
+  <dimension ref="A2:E42"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="6.33203125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="53.4140625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="67.9140625" style="8" customWidth="1"/>
     <col min="3" max="4" width="13" style="17" customWidth="1"/>
     <col min="5" max="5" width="48.08203125" style="2" customWidth="1"/>
     <col min="6" max="16384" width="8.6640625" style="2"/>
@@ -746,7 +767,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="38" customHeight="1">
+    <row r="8" spans="1:5" ht="37.5" customHeight="1">
       <c r="A8" s="11">
         <v>4</v>
       </c>
@@ -763,258 +784,258 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="33" customHeight="1">
-      <c r="A9" s="11">
+    <row r="9" spans="1:5" ht="123.5" customHeight="1">
+      <c r="A9" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="9">
+        <v>46296</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:5" ht="73.5" customHeight="1">
+      <c r="A10" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="9">
+        <v>46296</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="1:5" ht="33" customHeight="1">
+      <c r="A11" s="11">
         <v>5</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B11" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C11" s="9">
         <v>46274</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D11" s="9">
         <v>46280</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="51.5" customHeight="1">
-      <c r="A10" s="11">
+    <row r="12" spans="1:5" ht="51.5" customHeight="1">
+      <c r="A12" s="11">
         <v>6</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B12" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C12" s="9">
         <v>46274</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D12" s="9">
         <v>46280</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="45.5" customHeight="1">
-      <c r="A11" s="11">
+    <row r="13" spans="1:5" ht="45.5" customHeight="1">
+      <c r="A13" s="11">
         <v>7</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B13" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C13" s="9">
         <v>46296</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D13" s="9">
         <v>46310</v>
       </c>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="1:5" ht="20" customHeight="1">
-      <c r="A12" s="11">
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" ht="20" customHeight="1">
+      <c r="A14" s="11">
         <v>8</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B14" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="21">
+      <c r="C14" s="21">
         <v>46274</v>
       </c>
-      <c r="D12" s="21">
+      <c r="D14" s="21">
         <v>46290</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="20" customHeight="1">
-      <c r="A13" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="9">
-        <v>46274</v>
-      </c>
-      <c r="D13" s="9">
-        <v>46281</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="20" customHeight="1">
-      <c r="A14" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="9">
-        <v>46280</v>
-      </c>
-      <c r="D14" s="9">
-        <v>46281</v>
-      </c>
       <c r="E14" s="1" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="20" customHeight="1">
       <c r="A15" s="12" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C15" s="9">
-        <v>46276</v>
+        <v>46274</v>
       </c>
       <c r="D15" s="9">
-        <v>46289</v>
+        <v>46281</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="20" customHeight="1">
-      <c r="A16" s="11">
-        <v>9</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="20">
-        <f>C17</f>
-        <v>46277</v>
-      </c>
-      <c r="D16" s="20">
-        <v>46320</v>
-      </c>
-      <c r="E16" s="1"/>
+      <c r="A16" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="9">
+        <v>46280</v>
+      </c>
+      <c r="D16" s="9">
+        <v>46281</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="17" spans="1:5" ht="20" customHeight="1">
-      <c r="A17" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C17" s="6">
-        <v>46277</v>
-      </c>
-      <c r="D17" s="6">
-        <v>46290</v>
+      <c r="A17" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="9">
+        <v>46276</v>
+      </c>
+      <c r="D17" s="9">
+        <v>46289</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="20" customHeight="1">
-      <c r="A18" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="6">
-        <v>46293</v>
-      </c>
-      <c r="D18" s="6">
-        <v>46296</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>44</v>
-      </c>
+      <c r="A18" s="11">
+        <v>9</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="20">
+        <f>C19</f>
+        <v>46277</v>
+      </c>
+      <c r="D18" s="20">
+        <v>46320</v>
+      </c>
+      <c r="E18" s="1"/>
     </row>
     <row r="19" spans="1:5" ht="20" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="C19" s="6">
-        <v>46293</v>
+        <v>46277</v>
       </c>
       <c r="D19" s="6">
-        <v>46320</v>
+        <v>46290</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="20" customHeight="1">
       <c r="A20" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B20" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="20">
-        <v>46286</v>
-      </c>
-      <c r="D20" s="20">
-        <v>46318</v>
-      </c>
-      <c r="E20" s="1"/>
+        <v>50</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="6">
+        <v>46293</v>
+      </c>
+      <c r="D20" s="6">
+        <v>46296</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="21" spans="1:5" ht="20" customHeight="1">
       <c r="A21" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="6">
+        <v>46293</v>
+      </c>
+      <c r="D21" s="6">
+        <v>46320</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="20" customHeight="1">
+      <c r="A22" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="20">
+        <v>46286</v>
+      </c>
+      <c r="D22" s="20">
+        <v>46318</v>
+      </c>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:5" ht="20" customHeight="1">
+      <c r="A23" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B23" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C23" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D23" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="20" customHeight="1">
-      <c r="A22" s="4" t="s">
+      <c r="E23" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="20" customHeight="1">
+      <c r="A24" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="C22" s="6">
-        <v>46286</v>
-      </c>
-      <c r="D22" s="6">
-        <v>46307</v>
-      </c>
-      <c r="E22" s="1"/>
-    </row>
-    <row r="23" spans="1:5" ht="20" customHeight="1">
-      <c r="A23" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" s="6">
-        <v>46286</v>
-      </c>
-      <c r="D23" s="6">
-        <v>46307</v>
-      </c>
-      <c r="E23" s="1"/>
-    </row>
-    <row r="24" spans="1:5" ht="33.5" customHeight="1">
-      <c r="A24" s="4" t="s">
-        <v>55</v>
-      </c>
       <c r="B24" s="19" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="C24" s="6">
         <v>46286</v>
@@ -1026,120 +1047,120 @@
     </row>
     <row r="25" spans="1:5" ht="20" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="B25" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="6">
+        <v>46286</v>
+      </c>
+      <c r="D25" s="6">
+        <v>46307</v>
+      </c>
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="1:5" ht="33.5" customHeight="1">
+      <c r="A26" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="6">
+        <v>46286</v>
+      </c>
+      <c r="D26" s="6">
+        <v>46307</v>
+      </c>
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" spans="1:5" ht="20" customHeight="1">
+      <c r="A27" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="6">
+      <c r="C27" s="6">
         <v>46296</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D27" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E25" s="1"/>
-    </row>
-    <row r="26" spans="1:5" ht="36" customHeight="1">
-      <c r="A26" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="36" customHeight="1">
-      <c r="A27" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B27" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="C27" s="6">
-        <v>46311</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E27" s="5"/>
+      <c r="E27" s="1"/>
     </row>
     <row r="28" spans="1:5" ht="36" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="C28" s="6">
-        <v>46315</v>
-      </c>
-      <c r="D28" s="6">
-        <v>46317</v>
-      </c>
-      <c r="E28" s="5"/>
+        <v>13</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="29" spans="1:5" ht="36" customHeight="1">
       <c r="A29" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C29" s="6">
-        <v>46314</v>
-      </c>
-      <c r="D29" s="6">
-        <v>46317</v>
+        <v>46311</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="E29" s="5"/>
     </row>
     <row r="30" spans="1:5" ht="36" customHeight="1">
       <c r="A30" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C30" s="6">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="D30" s="6">
-        <v>46318</v>
+        <v>46317</v>
       </c>
       <c r="E30" s="5"/>
     </row>
     <row r="31" spans="1:5" ht="36" customHeight="1">
       <c r="A31" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="C31" s="6">
-        <v>46318</v>
+        <v>46314</v>
       </c>
       <c r="D31" s="6">
-        <v>46318</v>
+        <v>46317</v>
       </c>
       <c r="E31" s="5"/>
     </row>
     <row r="32" spans="1:5" ht="36" customHeight="1">
       <c r="A32" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C32" s="6">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="D32" s="6">
         <v>46318</v>
@@ -1147,68 +1168,98 @@
       <c r="E32" s="5"/>
     </row>
     <row r="33" spans="1:5" ht="36" customHeight="1">
-      <c r="A33" s="13">
+      <c r="A33" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" s="6">
+        <v>46318</v>
+      </c>
+      <c r="D33" s="6">
+        <v>46318</v>
+      </c>
+      <c r="E33" s="5"/>
+    </row>
+    <row r="34" spans="1:5" ht="36" customHeight="1">
+      <c r="A34" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B34" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="6">
+        <v>46318</v>
+      </c>
+      <c r="D34" s="6">
+        <v>46318</v>
+      </c>
+      <c r="E34" s="5"/>
+    </row>
+    <row r="35" spans="1:5" ht="36" customHeight="1">
+      <c r="A35" s="13">
         <v>11</v>
       </c>
-      <c r="B33" s="18" t="s">
+      <c r="B35" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C33" s="16">
+      <c r="C35" s="16">
         <v>46318</v>
       </c>
-      <c r="D33" s="16">
+      <c r="D35" s="16">
         <v>46318</v>
       </c>
-      <c r="E33" s="5"/>
-    </row>
-    <row r="34" spans="1:5" ht="36" customHeight="1">
-      <c r="A34" s="13">
+      <c r="E35" s="5"/>
+    </row>
+    <row r="36" spans="1:5" ht="36" customHeight="1">
+      <c r="A36" s="13">
         <v>12</v>
       </c>
-      <c r="B34" s="18" t="s">
+      <c r="B36" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="C34" s="16">
+      <c r="C36" s="16">
         <v>46320</v>
       </c>
-      <c r="D34" s="16">
+      <c r="D36" s="16">
         <v>46320</v>
       </c>
-      <c r="E34" s="5"/>
-    </row>
-    <row r="35" spans="1:5" ht="36" customHeight="1">
-      <c r="B35" s="18"/>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="5"/>
-    </row>
-    <row r="36" spans="1:5" ht="36" customHeight="1">
-      <c r="B36" s="18"/>
-      <c r="C36" s="16"/>
-      <c r="D36" s="16"/>
       <c r="E36" s="5"/>
     </row>
     <row r="37" spans="1:5" ht="36" customHeight="1">
-      <c r="A37" s="4"/>
-      <c r="B37" s="5"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
       <c r="E37" s="5"/>
     </row>
     <row r="38" spans="1:5" ht="36" customHeight="1">
-      <c r="A38" s="4"/>
-      <c r="B38" s="5"/>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
       <c r="E38" s="5"/>
     </row>
-    <row r="39" spans="1:5">
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
-    </row>
-    <row r="40" spans="1:5">
-      <c r="C40" s="16"/>
-      <c r="D40" s="16"/>
+    <row r="39" spans="1:5" ht="36" customHeight="1">
+      <c r="A39" s="4"/>
+      <c r="B39" s="5"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="5"/>
+    </row>
+    <row r="40" spans="1:5" ht="36" customHeight="1">
+      <c r="A40" s="4"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="5"/>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="C42" s="16"/>
+      <c r="D42" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Update schedule and record budget approval on October 13
</commit_message>
<xml_diff>
--- a/dist/График_подготовки_Октоберфест.xlsx
+++ b/dist/График_подготовки_Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B3F3416-0197-4FFD-B78C-E2F9EAF76D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E155D5-72A1-4EA3-B271-5B4CFF562C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -222,9 +222,6 @@
     <t>10.12.</t>
   </si>
   <si>
-    <t>выполнено частично. Получены замечания к Бюджету</t>
-  </si>
-  <si>
     <t>4.1.</t>
   </si>
   <si>
@@ -253,6 +250,9 @@
   </si>
   <si>
     <t>заказ оформлен. Ожидается поставка</t>
+  </si>
+  <si>
+    <t>выполнено. Согласован В.Ксенофонтовым 13.10.26</t>
   </si>
 </sst>
 </file>
@@ -796,31 +796,31 @@
     </row>
     <row r="9" spans="1:5" ht="36" customHeight="1">
       <c r="A9" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C9" s="9">
         <v>46296</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" ht="59" customHeight="1">
       <c r="A10" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C10" s="9">
         <v>46296</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E10" s="1"/>
     </row>
@@ -873,7 +873,7 @@
       </c>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:5" ht="20" customHeight="1">
+    <row r="14" spans="1:5" ht="34.5" customHeight="1">
       <c r="A14" s="11">
         <v>8</v>
       </c>
@@ -886,8 +886,8 @@
       <c r="D14" s="21">
         <v>46290</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>62</v>
+      <c r="E14" s="7" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="20" customHeight="1">
@@ -1037,7 +1037,7 @@
         <v>8</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="20" customHeight="1">
@@ -1054,7 +1054,7 @@
         <v>46307</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="20" customHeight="1">
@@ -1071,7 +1071,7 @@
         <v>46307</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="33.5" customHeight="1">
@@ -1088,7 +1088,7 @@
         <v>46307</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="20" customHeight="1">
@@ -1105,7 +1105,7 @@
         <v>12</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="36" customHeight="1">

</xml_diff>

<commit_message>
Refresh Oktoberfest schedule for 16 October
</commit_message>
<xml_diff>
--- a/dist/График_подготовки_Октоберфест.xlsx
+++ b/dist/График_подготовки_Октоберфест.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E155D5-72A1-4EA3-B271-5B4CFF562C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{282F6880-AB8D-45D5-9707-39A04FBCA840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="График" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="74">
   <si>
     <t>График подготовки к фестивалю Октоберфест</t>
   </si>
@@ -138,9 +138,6 @@
   </si>
   <si>
     <t>Определить локации проведения фестиваля (предусмтореть погодные условия)</t>
-  </si>
-  <si>
-    <t>Подготовить детальное ценообразование по фуд/гриль/лаунж зонам</t>
   </si>
   <si>
     <t>Определить и утвердить локации для проведения фудовых и тематических мастер-классов и активностей, их количество и варианты</t>
@@ -253,6 +250,15 @@
   </si>
   <si>
     <t>выполнено. Согласован В.Ксенофонтовым 13.10.26</t>
+  </si>
+  <si>
+    <t>Подготовить детальное ценообразование по фуд/гриль зонам</t>
+  </si>
+  <si>
+    <t>на продукцию сформирован. На пиво 16.10.26</t>
+  </si>
+  <si>
+    <t>частично получено</t>
   </si>
 </sst>
 </file>
@@ -740,7 +746,7 @@
         <v>46276</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="33.5" customHeight="1">
@@ -757,7 +763,7 @@
         <v>46280</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="20" customHeight="1">
@@ -774,7 +780,7 @@
         <v>46280</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="37.5" customHeight="1">
@@ -791,36 +797,36 @@
         <v>46280</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="36" customHeight="1">
       <c r="A9" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C9" s="9">
         <v>46296</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" ht="59" customHeight="1">
       <c r="A10" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C10" s="9">
         <v>46296</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E10" s="1"/>
     </row>
@@ -838,7 +844,7 @@
         <v>46280</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="51.5" customHeight="1">
@@ -846,7 +852,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C12" s="9">
         <v>46274</v>
@@ -855,7 +861,7 @@
         <v>46280</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="45.5" customHeight="1">
@@ -863,7 +869,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="C13" s="9">
         <v>46296</v>
@@ -887,12 +893,12 @@
         <v>46290</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="20" customHeight="1">
       <c r="A15" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B15" s="22" t="s">
         <v>26</v>
@@ -904,12 +910,12 @@
         <v>46281</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="20" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B16" s="22" t="s">
         <v>27</v>
@@ -921,12 +927,12 @@
         <v>46281</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="20" customHeight="1">
       <c r="A17" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B17" s="22" t="s">
         <v>28</v>
@@ -938,7 +944,7 @@
         <v>46289</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="20" customHeight="1">
@@ -959,7 +965,7 @@
     </row>
     <row r="19" spans="1:5" ht="20" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>20</v>
@@ -971,12 +977,12 @@
         <v>46290</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="20" customHeight="1">
       <c r="A20" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>21</v>
@@ -988,15 +994,15 @@
         <v>46296</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="20" customHeight="1">
       <c r="A21" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21" s="6">
         <v>46293</v>
@@ -1005,12 +1011,12 @@
         <v>46320</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="20" customHeight="1">
       <c r="A22" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>29</v>
@@ -1025,7 +1031,7 @@
     </row>
     <row r="23" spans="1:5" ht="20" customHeight="1">
       <c r="A23" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B23" s="19" t="s">
         <v>6</v>
@@ -1037,15 +1043,15 @@
         <v>8</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="20" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C24" s="6">
         <v>46286</v>
@@ -1054,12 +1060,12 @@
         <v>46307</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="20" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B25" s="19" t="s">
         <v>9</v>
@@ -1071,12 +1077,12 @@
         <v>46307</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="33.5" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>10</v>
@@ -1088,12 +1094,12 @@
         <v>46307</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="20" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B27" s="19" t="s">
         <v>11</v>
@@ -1105,12 +1111,12 @@
         <v>12</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="36" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B28" s="19" t="s">
         <v>13</v>
@@ -1122,12 +1128,12 @@
         <v>12</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="36" customHeight="1">
       <c r="A29" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B29" s="19" t="s">
         <v>14</v>
@@ -1138,11 +1144,13 @@
       <c r="D29" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="5"/>
+      <c r="E29" s="5" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="30" spans="1:5" ht="36" customHeight="1">
       <c r="A30" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B30" s="19" t="s">
         <v>17</v>
@@ -1157,7 +1165,7 @@
     </row>
     <row r="31" spans="1:5" ht="36" customHeight="1">
       <c r="A31" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B31" s="19" t="s">
         <v>16</v>
@@ -1168,11 +1176,13 @@
       <c r="D31" s="6">
         <v>46317</v>
       </c>
-      <c r="E31" s="5"/>
+      <c r="E31" s="5" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="32" spans="1:5" ht="36" customHeight="1">
       <c r="A32" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B32" s="19" t="s">
         <v>22</v>
@@ -1187,10 +1197,10 @@
     </row>
     <row r="33" spans="1:5" ht="36" customHeight="1">
       <c r="A33" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C33" s="6">
         <v>46318</v>
@@ -1202,7 +1212,7 @@
     </row>
     <row r="34" spans="1:5" ht="36" customHeight="1">
       <c r="A34" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B34" s="19" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Revert "Refresh Oktoberfest schedule for 16 October"
This reverts commit 99d583cf186fd0e75739b6ae8da43d641391c3d4.
</commit_message>
<xml_diff>
--- a/dist/График_подготовки_Октоберфест.xlsx
+++ b/dist/График_подготовки_Октоберфест.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{282F6880-AB8D-45D5-9707-39A04FBCA840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E155D5-72A1-4EA3-B271-5B4CFF562C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="График" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="72">
   <si>
     <t>График подготовки к фестивалю Октоберфест</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>Определить локации проведения фестиваля (предусмтореть погодные условия)</t>
+  </si>
+  <si>
+    <t>Подготовить детальное ценообразование по фуд/гриль/лаунж зонам</t>
   </si>
   <si>
     <t>Определить и утвердить локации для проведения фудовых и тематических мастер-классов и активностей, их количество и варианты</t>
@@ -250,15 +253,6 @@
   </si>
   <si>
     <t>выполнено. Согласован В.Ксенофонтовым 13.10.26</t>
-  </si>
-  <si>
-    <t>Подготовить детальное ценообразование по фуд/гриль зонам</t>
-  </si>
-  <si>
-    <t>на продукцию сформирован. На пиво 16.10.26</t>
-  </si>
-  <si>
-    <t>частично получено</t>
   </si>
 </sst>
 </file>
@@ -746,7 +740,7 @@
         <v>46276</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="33.5" customHeight="1">
@@ -763,7 +757,7 @@
         <v>46280</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="20" customHeight="1">
@@ -780,7 +774,7 @@
         <v>46280</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="37.5" customHeight="1">
@@ -797,36 +791,36 @@
         <v>46280</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="36" customHeight="1">
       <c r="A9" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C9" s="9">
         <v>46296</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" ht="59" customHeight="1">
       <c r="A10" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C10" s="9">
         <v>46296</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E10" s="1"/>
     </row>
@@ -844,7 +838,7 @@
         <v>46280</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="51.5" customHeight="1">
@@ -852,7 +846,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C12" s="9">
         <v>46274</v>
@@ -861,7 +855,7 @@
         <v>46280</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="45.5" customHeight="1">
@@ -869,7 +863,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="C13" s="9">
         <v>46296</v>
@@ -893,12 +887,12 @@
         <v>46290</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="20" customHeight="1">
       <c r="A15" s="12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B15" s="22" t="s">
         <v>26</v>
@@ -910,12 +904,12 @@
         <v>46281</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="20" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B16" s="22" t="s">
         <v>27</v>
@@ -927,12 +921,12 @@
         <v>46281</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="20" customHeight="1">
       <c r="A17" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B17" s="22" t="s">
         <v>28</v>
@@ -944,7 +938,7 @@
         <v>46289</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="20" customHeight="1">
@@ -965,7 +959,7 @@
     </row>
     <row r="19" spans="1:5" ht="20" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>20</v>
@@ -977,12 +971,12 @@
         <v>46290</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="20" customHeight="1">
       <c r="A20" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>21</v>
@@ -994,15 +988,15 @@
         <v>46296</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="20" customHeight="1">
       <c r="A21" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C21" s="6">
         <v>46293</v>
@@ -1011,12 +1005,12 @@
         <v>46320</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="20" customHeight="1">
       <c r="A22" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>29</v>
@@ -1031,7 +1025,7 @@
     </row>
     <row r="23" spans="1:5" ht="20" customHeight="1">
       <c r="A23" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B23" s="19" t="s">
         <v>6</v>
@@ -1043,15 +1037,15 @@
         <v>8</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="20" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C24" s="6">
         <v>46286</v>
@@ -1060,12 +1054,12 @@
         <v>46307</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="20" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B25" s="19" t="s">
         <v>9</v>
@@ -1077,12 +1071,12 @@
         <v>46307</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="33.5" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>10</v>
@@ -1094,12 +1088,12 @@
         <v>46307</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="20" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B27" s="19" t="s">
         <v>11</v>
@@ -1111,12 +1105,12 @@
         <v>12</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="36" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B28" s="19" t="s">
         <v>13</v>
@@ -1128,12 +1122,12 @@
         <v>12</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="36" customHeight="1">
       <c r="A29" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B29" s="19" t="s">
         <v>14</v>
@@ -1144,13 +1138,11 @@
       <c r="D29" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="5" t="s">
-        <v>72</v>
-      </c>
+      <c r="E29" s="5"/>
     </row>
     <row r="30" spans="1:5" ht="36" customHeight="1">
       <c r="A30" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B30" s="19" t="s">
         <v>17</v>
@@ -1165,7 +1157,7 @@
     </row>
     <row r="31" spans="1:5" ht="36" customHeight="1">
       <c r="A31" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B31" s="19" t="s">
         <v>16</v>
@@ -1176,13 +1168,11 @@
       <c r="D31" s="6">
         <v>46317</v>
       </c>
-      <c r="E31" s="5" t="s">
-        <v>73</v>
-      </c>
+      <c r="E31" s="5"/>
     </row>
     <row r="32" spans="1:5" ht="36" customHeight="1">
       <c r="A32" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B32" s="19" t="s">
         <v>22</v>
@@ -1197,10 +1187,10 @@
     </row>
     <row r="33" spans="1:5" ht="36" customHeight="1">
       <c r="A33" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C33" s="6">
         <v>46318</v>
@@ -1212,7 +1202,7 @@
     </row>
     <row r="34" spans="1:5" ht="36" customHeight="1">
       <c r="A34" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B34" s="19" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Sync updated Oktoberfest schedule
</commit_message>
<xml_diff>
--- a/dist/График_подготовки_Октоберфест.xlsx
+++ b/dist/График_подготовки_Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82684E96-AFD3-47B4-929A-49F07E509B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA840A5-124A-47FF-A838-E2BB582F6265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="76">
   <si>
     <t>График подготовки к фестивалю Октоберфест</t>
   </si>
@@ -246,12 +246,6 @@
     <t>В процессе согласования</t>
   </si>
   <si>
-    <t>заказ оформлен. Ожидается поставка</t>
-  </si>
-  <si>
-    <t>выполнено. Согласован В.Ксенофонтовым 13.10.26</t>
-  </si>
-  <si>
     <t>Подготовить детальное ценообразование по фуд/гриль зонам</t>
   </si>
   <si>
@@ -261,10 +255,16 @@
     <t>частично получено</t>
   </si>
   <si>
-    <t>будет 16.10.26</t>
-  </si>
-  <si>
     <t>выполнено. Требуется корректировка локаций с учетом строительства катка</t>
+  </si>
+  <si>
+    <t>выполнено. Согласован В.Ксенофонтовым 13.10.26. Ожидается согласование Н.Луканихиной</t>
+  </si>
+  <si>
+    <t>заказ оформлен. Ожидается поставка 21.10.26</t>
+  </si>
+  <si>
+    <t>выполнено. Лофт и "Семейная зона"</t>
   </si>
 </sst>
 </file>
@@ -335,7 +335,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -405,7 +405,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -474,6 +474,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -481,9 +487,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -715,13 +718,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" ht="24" customHeight="1">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="26"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="28"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="11"/>
@@ -828,7 +831,9 @@
       <c r="D9" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="1"/>
+      <c r="E9" s="1" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="10" spans="1:5" ht="59" customHeight="1">
       <c r="A10" s="11" t="s">
@@ -843,7 +848,9 @@
       <c r="D10" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="E10" s="1"/>
+      <c r="E10" s="1" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="11" spans="1:5" ht="33" customHeight="1">
       <c r="A11" s="11">
@@ -859,7 +866,7 @@
         <v>46280</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>41</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="51.5" customHeight="1">
@@ -876,7 +883,7 @@
         <v>46280</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="45.5" customHeight="1">
@@ -884,7 +891,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C13" s="9">
         <v>46296</v>
@@ -893,7 +900,7 @@
         <v>46310</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="34.5" customHeight="1">
@@ -910,7 +917,7 @@
         <v>46290</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="20" customHeight="1">
@@ -1081,10 +1088,10 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="20" customHeight="1">
-      <c r="A25" s="27" t="s">
+      <c r="A25" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="24" t="s">
         <v>9</v>
       </c>
       <c r="C25" s="6">
@@ -1093,12 +1100,12 @@
       <c r="D25" s="6">
         <v>46307</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="E25" s="25" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="33.5" customHeight="1">
-      <c r="A26" s="27" t="s">
+      <c r="A26" s="4" t="s">
         <v>52</v>
       </c>
       <c r="B26" s="19" t="s">
@@ -1115,10 +1122,10 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="20" customHeight="1">
-      <c r="A27" s="27" t="s">
+      <c r="A27" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="24" t="s">
         <v>11</v>
       </c>
       <c r="C27" s="6">
@@ -1127,8 +1134,8 @@
       <c r="D27" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>69</v>
+      <c r="E27" s="25" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="36" customHeight="1">
@@ -1149,7 +1156,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="36" customHeight="1">
-      <c r="A29" s="27" t="s">
+      <c r="A29" s="4" t="s">
         <v>55</v>
       </c>
       <c r="B29" s="19" t="s">
@@ -1162,7 +1169,7 @@
         <v>15</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="36" customHeight="1">
@@ -1194,7 +1201,7 @@
         <v>46317</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="36" customHeight="1">

</xml_diff>

<commit_message>
Sync October schedule and timing
</commit_message>
<xml_diff>
--- a/dist/График_подготовки_Октоберфест.xlsx
+++ b/dist/График_подготовки_Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA840A5-124A-47FF-A838-E2BB582F6265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{764FEBBE-A28F-4E3C-AD4F-560F2F733B26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="72">
   <si>
     <t>График подготовки к фестивалю Октоберфест</t>
   </si>
@@ -160,9 +160,6 @@
   </si>
   <si>
     <t>выполнено</t>
-  </si>
-  <si>
-    <t>выполнено 28.09.26</t>
   </si>
   <si>
     <t>Поиск диджея и заключение договора</t>
@@ -240,31 +237,22 @@
 </t>
   </si>
   <si>
-    <t>Ожидается договор от Контрагента. 13.10.26</t>
-  </si>
-  <si>
     <t>В процессе согласования</t>
   </si>
   <si>
     <t>Подготовить детальное ценообразование по фуд/гриль зонам</t>
   </si>
   <si>
-    <t>на продукцию сформирован. На пиво 16.10.26</t>
-  </si>
-  <si>
     <t>частично получено</t>
   </si>
   <si>
-    <t>выполнено. Требуется корректировка локаций с учетом строительства катка</t>
-  </si>
-  <si>
     <t>выполнено. Согласован В.Ксенофонтовым 13.10.26. Ожидается согласование Н.Луканихиной</t>
   </si>
   <si>
-    <t>заказ оформлен. Ожидается поставка 21.10.26</t>
-  </si>
-  <si>
     <t>выполнено. Лофт и "Семейная зона"</t>
+  </si>
+  <si>
+    <t>выполнено. Согласно плану с таймингом</t>
   </si>
 </sst>
 </file>
@@ -321,7 +309,7 @@
       <charset val="204"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -331,12 +319,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -405,7 +387,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -474,12 +456,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -488,6 +464,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -718,13 +697,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" ht="24" customHeight="1">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="28"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="26"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="11"/>
@@ -820,16 +799,16 @@
     </row>
     <row r="9" spans="1:5" ht="36" customHeight="1">
       <c r="A9" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C9" s="9">
         <v>46296</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>41</v>
@@ -837,16 +816,16 @@
     </row>
     <row r="10" spans="1:5" ht="59" customHeight="1">
       <c r="A10" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C10" s="9">
         <v>46296</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>41</v>
@@ -866,7 +845,7 @@
         <v>46280</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="51.5" customHeight="1">
@@ -883,7 +862,7 @@
         <v>46280</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="45.5" customHeight="1">
@@ -891,7 +870,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C13" s="9">
         <v>46296</v>
@@ -917,12 +896,12 @@
         <v>46290</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="20" customHeight="1">
       <c r="A15" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B15" s="22" t="s">
         <v>26</v>
@@ -939,7 +918,7 @@
     </row>
     <row r="16" spans="1:5" ht="20" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B16" s="22" t="s">
         <v>27</v>
@@ -956,7 +935,7 @@
     </row>
     <row r="17" spans="1:5" ht="20" customHeight="1">
       <c r="A17" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B17" s="22" t="s">
         <v>28</v>
@@ -989,7 +968,7 @@
     </row>
     <row r="19" spans="1:5" ht="20" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>20</v>
@@ -1006,7 +985,7 @@
     </row>
     <row r="20" spans="1:5" ht="20" customHeight="1">
       <c r="A20" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>21</v>
@@ -1018,12 +997,12 @@
         <v>46296</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="20" customHeight="1">
       <c r="A21" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>40</v>
@@ -1035,12 +1014,12 @@
         <v>46320</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="20" customHeight="1">
       <c r="A22" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>29</v>
@@ -1067,7 +1046,7 @@
         <v>8</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="20" customHeight="1">
@@ -1075,7 +1054,7 @@
         <v>37</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C24" s="6">
         <v>46286</v>
@@ -1084,14 +1063,14 @@
         <v>46307</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="20" customHeight="1">
       <c r="A25" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="27" t="s">
         <v>9</v>
       </c>
       <c r="C25" s="6">
@@ -1100,13 +1079,13 @@
       <c r="D25" s="6">
         <v>46307</v>
       </c>
-      <c r="E25" s="25" t="s">
-        <v>67</v>
+      <c r="E25" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="33.5" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>10</v>
@@ -1118,14 +1097,14 @@
         <v>46307</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="20" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B27" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="27" t="s">
         <v>11</v>
       </c>
       <c r="C27" s="6">
@@ -1134,13 +1113,13 @@
       <c r="D27" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E27" s="25" t="s">
-        <v>74</v>
+      <c r="E27" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="36" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B28" s="19" t="s">
         <v>13</v>
@@ -1157,7 +1136,7 @@
     </row>
     <row r="29" spans="1:5" ht="36" customHeight="1">
       <c r="A29" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B29" s="19" t="s">
         <v>14</v>
@@ -1169,12 +1148,12 @@
         <v>15</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="36" customHeight="1">
       <c r="A30" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B30" s="19" t="s">
         <v>17</v>
@@ -1189,7 +1168,7 @@
     </row>
     <row r="31" spans="1:5" ht="36" customHeight="1">
       <c r="A31" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B31" s="19" t="s">
         <v>16</v>
@@ -1201,12 +1180,12 @@
         <v>46317</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="36" customHeight="1">
       <c r="A32" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B32" s="19" t="s">
         <v>22</v>
@@ -1221,7 +1200,7 @@
     </row>
     <row r="33" spans="1:5" ht="36" customHeight="1">
       <c r="A33" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B33" s="19" t="s">
         <v>39</v>
@@ -1236,7 +1215,7 @@
     </row>
     <row r="34" spans="1:5" ht="36" customHeight="1">
       <c r="A34" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B34" s="19" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Sync Oktoberfest schedule and timing
</commit_message>
<xml_diff>
--- a/dist/График_подготовки_Октоберфест.xlsx
+++ b/dist/График_подготовки_Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{764FEBBE-A28F-4E3C-AD4F-560F2F733B26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A5EE863-1EE9-4B76-8633-E2FB1369CF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
   <si>
     <t>График подготовки к фестивалю Октоберфест</t>
   </si>
@@ -65,12 +65,6 @@
     <t>Заключить договор аренды звукового и светового оборудования</t>
   </si>
   <si>
-    <t>При необходимости обновить договоры с ведущими и аниматорами</t>
-  </si>
-  <si>
-    <t>Закупить материалы для мастер-классов</t>
-  </si>
-  <si>
     <t>15.10.2026</t>
   </si>
   <si>
@@ -84,9 +78,6 @@
   </si>
   <si>
     <t>Прием поставки продукции в парк</t>
-  </si>
-  <si>
-    <t>Установка звукового и светового оборудования на сцене</t>
   </si>
   <si>
     <t>Проверка готовности. Развоз ингредиентов и продукции. Установка кег с пивом</t>
@@ -237,22 +228,37 @@
 </t>
   </si>
   <si>
-    <t>В процессе согласования</t>
-  </si>
-  <si>
     <t>Подготовить детальное ценообразование по фуд/гриль зонам</t>
   </si>
   <si>
     <t>частично получено</t>
   </si>
   <si>
-    <t>выполнено. Согласован В.Ксенофонтовым 13.10.26. Ожидается согласование Н.Луканихиной</t>
-  </si>
-  <si>
     <t>выполнено. Лофт и "Семейная зона"</t>
   </si>
   <si>
     <t>выполнено. Согласно плану с таймингом</t>
+  </si>
+  <si>
+    <t>Обновить договоры с ведущими и аниматорами</t>
+  </si>
+  <si>
+    <t>В работе. Договоры проходят процедуру согласования в ПС</t>
+  </si>
+  <si>
+    <t>выполнено. Согласован В.Ксенофонтовым 13.10.26. Ожидается согласование Н.Луканихиной 20.10.26</t>
+  </si>
+  <si>
+    <t>Закупить материалы для мастер-классов, костюмы для анимации, гирлянды, арендовать бочки</t>
+  </si>
+  <si>
+    <t>Установка звукового и светового оборудования в Лофте</t>
+  </si>
+  <si>
+    <t>Выполнено. 23.10.26 Ожидается поставка бочек и гирлянды</t>
+  </si>
+  <si>
+    <t>20.10.26 будет тест экрана</t>
   </si>
 </sst>
 </file>
@@ -387,7 +393,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -414,9 +420,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -453,9 +456,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -465,7 +465,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -688,28 +688,28 @@
   <dimension ref="A2:E42"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="6.33203125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="67.9140625" style="8" customWidth="1"/>
-    <col min="3" max="4" width="13" style="17" customWidth="1"/>
+    <col min="1" max="1" width="6.33203125" style="12" customWidth="1"/>
+    <col min="2" max="2" width="69.33203125" style="8" customWidth="1"/>
+    <col min="3" max="4" width="13" style="16" customWidth="1"/>
     <col min="5" max="5" width="48.08203125" style="2" customWidth="1"/>
     <col min="6" max="6" width="30" style="2" customWidth="1"/>
     <col min="7" max="16384" width="8.6640625" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:5" ht="24" customHeight="1">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="26"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="24"/>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="11"/>
+      <c r="A3" s="10"/>
       <c r="B3" s="7"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1">
@@ -730,11 +730,11 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="26.5" customHeight="1">
-      <c r="A5" s="11">
+      <c r="A5" s="10">
         <v>1</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>30</v>
+      <c r="B5" s="25" t="s">
+        <v>27</v>
       </c>
       <c r="C5" s="9">
         <v>46274</v>
@@ -743,15 +743,15 @@
         <v>46276</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="33.5" customHeight="1">
-      <c r="A6" s="11">
+      <c r="A6" s="10">
         <v>2</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>31</v>
+      <c r="B6" s="25" t="s">
+        <v>28</v>
       </c>
       <c r="C6" s="9">
         <v>46274</v>
@@ -760,15 +760,15 @@
         <v>46280</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="20" customHeight="1">
-      <c r="A7" s="11">
+      <c r="A7" s="10">
         <v>3</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>32</v>
+      <c r="B7" s="25" t="s">
+        <v>29</v>
       </c>
       <c r="C7" s="9">
         <v>46274</v>
@@ -777,15 +777,15 @@
         <v>46280</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="37.5" customHeight="1">
-      <c r="A8" s="11">
+      <c r="A8" s="10">
         <v>4</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>33</v>
+      <c r="B8" s="25" t="s">
+        <v>30</v>
       </c>
       <c r="C8" s="9">
         <v>46274</v>
@@ -794,49 +794,49 @@
         <v>46280</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="36" customHeight="1">
-      <c r="A9" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>65</v>
+      <c r="A9" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>62</v>
       </c>
       <c r="C9" s="9">
         <v>46296</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="59" customHeight="1">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="25" t="s">
         <v>61</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>64</v>
       </c>
       <c r="C10" s="9">
         <v>46296</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="33" customHeight="1">
-      <c r="A11" s="11">
+      <c r="A11" s="10">
         <v>5</v>
       </c>
-      <c r="B11" s="15" t="s">
-        <v>34</v>
+      <c r="B11" s="25" t="s">
+        <v>31</v>
       </c>
       <c r="C11" s="9">
         <v>46274</v>
@@ -845,15 +845,15 @@
         <v>46280</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="51.5" customHeight="1">
-      <c r="A12" s="11">
+      <c r="A12" s="10">
         <v>6</v>
       </c>
-      <c r="B12" s="15" t="s">
-        <v>35</v>
+      <c r="B12" s="25" t="s">
+        <v>32</v>
       </c>
       <c r="C12" s="9">
         <v>46274</v>
@@ -862,15 +862,15 @@
         <v>46280</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="45.5" customHeight="1">
-      <c r="A13" s="11">
+      <c r="A13" s="10">
         <v>7</v>
       </c>
-      <c r="B13" s="15" t="s">
-        <v>67</v>
+      <c r="B13" s="25" t="s">
+        <v>63</v>
       </c>
       <c r="C13" s="9">
         <v>46296</v>
@@ -879,20 +879,20 @@
         <v>46310</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="34.5" customHeight="1">
-      <c r="A14" s="11">
+      <c r="A14" s="10">
         <v>8</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="21">
+      <c r="B14" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="20">
         <v>46274</v>
       </c>
-      <c r="D14" s="21">
+      <c r="D14" s="20">
         <v>46290</v>
       </c>
       <c r="E14" s="7" t="s">
@@ -900,11 +900,11 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="20" customHeight="1">
-      <c r="A15" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" s="22" t="s">
-        <v>26</v>
+      <c r="A15" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>23</v>
       </c>
       <c r="C15" s="9">
         <v>46274</v>
@@ -913,15 +913,15 @@
         <v>46281</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="20" customHeight="1">
-      <c r="A16" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>27</v>
+      <c r="A16" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>24</v>
       </c>
       <c r="C16" s="9">
         <v>46280</v>
@@ -930,15 +930,15 @@
         <v>46281</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="20" customHeight="1">
-      <c r="A17" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="22" t="s">
-        <v>28</v>
+      <c r="A17" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>25</v>
       </c>
       <c r="C17" s="9">
         <v>46276</v>
@@ -947,31 +947,31 @@
         <v>46289</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="20" customHeight="1">
-      <c r="A18" s="11">
+      <c r="A18" s="10">
         <v>9</v>
       </c>
-      <c r="B18" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="20">
+      <c r="B18" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="19">
         <f>C19</f>
         <v>46277</v>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="19">
         <v>46320</v>
       </c>
       <c r="E18" s="1"/>
     </row>
     <row r="19" spans="1:5" ht="20" customHeight="1">
-      <c r="A19" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>20</v>
+      <c r="A19" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>17</v>
       </c>
       <c r="C19" s="6">
         <v>46277</v>
@@ -980,15 +980,15 @@
         <v>46290</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="20" customHeight="1">
-      <c r="A20" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>21</v>
+      <c r="A20" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>18</v>
       </c>
       <c r="C20" s="6">
         <v>46293</v>
@@ -997,15 +997,15 @@
         <v>46296</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="20" customHeight="1">
-      <c r="A21" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>40</v>
+      <c r="A21" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>37</v>
       </c>
       <c r="C21" s="6">
         <v>46293</v>
@@ -1014,29 +1014,29 @@
         <v>46320</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="20" customHeight="1">
-      <c r="A22" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" s="20">
+      <c r="A22" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="19">
         <v>46286</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="19">
         <v>46318</v>
       </c>
       <c r="E22" s="1"/>
     </row>
     <row r="23" spans="1:5" ht="20" customHeight="1">
-      <c r="A23" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B23" s="19" t="s">
+      <c r="A23" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C23" s="6" t="s">
@@ -1045,16 +1045,16 @@
       <c r="D23" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E23" s="1" t="s">
-        <v>63</v>
+      <c r="E23" s="18" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="20" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B24" s="19" t="s">
-        <v>42</v>
+        <v>34</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>39</v>
       </c>
       <c r="C24" s="6">
         <v>46286</v>
@@ -1062,15 +1062,15 @@
       <c r="D24" s="6">
         <v>46307</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>63</v>
+      <c r="E24" s="18" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="20" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B25" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="18" t="s">
         <v>9</v>
       </c>
       <c r="C25" s="6">
@@ -1079,16 +1079,16 @@
       <c r="D25" s="6">
         <v>46307</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>63</v>
+      <c r="E25" s="18" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="33.5" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B26" s="19" t="s">
-        <v>10</v>
+        <v>48</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>67</v>
       </c>
       <c r="C26" s="6">
         <v>46286</v>
@@ -1096,67 +1096,67 @@
       <c r="D26" s="6">
         <v>46307</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="20" customHeight="1">
+      <c r="E26" s="18" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="30" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B27" s="27" t="s">
-        <v>11</v>
+        <v>49</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>70</v>
       </c>
       <c r="C27" s="6">
         <v>46296</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>63</v>
+        <v>10</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="36" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B28" s="19" t="s">
-        <v>13</v>
+        <v>50</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>11</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>41</v>
+        <v>10</v>
+      </c>
+      <c r="E28" s="18" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="36" customHeight="1">
       <c r="A29" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B29" s="19" t="s">
-        <v>14</v>
+        <v>51</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>12</v>
       </c>
       <c r="C29" s="6">
         <v>46311</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>41</v>
+        <v>13</v>
+      </c>
+      <c r="E29" s="18" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="36" customHeight="1">
       <c r="A30" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B30" s="19" t="s">
-        <v>17</v>
+        <v>52</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>71</v>
       </c>
       <c r="C30" s="6">
         <v>46315</v>
@@ -1164,14 +1164,16 @@
       <c r="D30" s="6">
         <v>46317</v>
       </c>
-      <c r="E30" s="5"/>
+      <c r="E30" s="5" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="31" spans="1:5" ht="36" customHeight="1">
       <c r="A31" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B31" s="19" t="s">
-        <v>16</v>
+        <v>53</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>14</v>
       </c>
       <c r="C31" s="6">
         <v>46314</v>
@@ -1180,15 +1182,15 @@
         <v>46317</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="36" customHeight="1">
       <c r="A32" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B32" s="19" t="s">
-        <v>22</v>
+        <v>54</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>19</v>
       </c>
       <c r="C32" s="6">
         <v>46316</v>
@@ -1200,10 +1202,10 @@
     </row>
     <row r="33" spans="1:5" ht="36" customHeight="1">
       <c r="A33" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B33" s="19" t="s">
-        <v>39</v>
+        <v>55</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>36</v>
       </c>
       <c r="C33" s="6">
         <v>46318</v>
@@ -1215,10 +1217,10 @@
     </row>
     <row r="34" spans="1:5" ht="36" customHeight="1">
       <c r="A34" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B34" s="19" t="s">
-        <v>18</v>
+        <v>56</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>15</v>
       </c>
       <c r="C34" s="6">
         <v>46318</v>
@@ -1229,45 +1231,45 @@
       <c r="E34" s="5"/>
     </row>
     <row r="35" spans="1:5" ht="24.5" customHeight="1">
-      <c r="A35" s="13">
+      <c r="A35" s="12">
         <v>11</v>
       </c>
-      <c r="B35" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C35" s="16">
+      <c r="B35" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="19">
         <v>46318</v>
       </c>
-      <c r="D35" s="16">
+      <c r="D35" s="19">
         <v>46318</v>
       </c>
       <c r="E35" s="5"/>
     </row>
     <row r="36" spans="1:5" ht="25.5" customHeight="1">
-      <c r="A36" s="13">
+      <c r="A36" s="12">
         <v>12</v>
       </c>
-      <c r="B36" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="C36" s="16">
+      <c r="B36" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="C36" s="19">
         <v>46320</v>
       </c>
-      <c r="D36" s="16">
+      <c r="D36" s="19">
         <v>46320</v>
       </c>
       <c r="E36" s="5"/>
     </row>
     <row r="37" spans="1:5" ht="36" customHeight="1">
-      <c r="B37" s="18"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
       <c r="E37" s="5"/>
     </row>
     <row r="38" spans="1:5" ht="36" customHeight="1">
-      <c r="B38" s="18"/>
-      <c r="C38" s="16"/>
-      <c r="D38" s="16"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
       <c r="E38" s="5"/>
     </row>
     <row r="39" spans="1:5" ht="36" customHeight="1">
@@ -1285,12 +1287,12 @@
       <c r="E40" s="5"/>
     </row>
     <row r="41" spans="1:5">
-      <c r="C41" s="16"/>
-      <c r="D41" s="16"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
     </row>
     <row r="42" spans="1:5">
-      <c r="C42" s="16"/>
-      <c r="D42" s="16"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Sync October festival task schedule
</commit_message>
<xml_diff>
--- a/dist/График_подготовки_Октоберфест.xlsx
+++ b/dist/График_подготовки_Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A5EE863-1EE9-4B76-8633-E2FB1369CF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2DCBF7D-21CD-4F99-A671-718CA9236E74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="70">
   <si>
     <t>График подготовки к фестивалю Октоберфест</t>
   </si>
@@ -231,9 +231,6 @@
     <t>Подготовить детальное ценообразование по фуд/гриль зонам</t>
   </si>
   <si>
-    <t>частично получено</t>
-  </si>
-  <si>
     <t>выполнено. Лофт и "Семейная зона"</t>
   </si>
   <si>
@@ -243,9 +240,6 @@
     <t>Обновить договоры с ведущими и аниматорами</t>
   </si>
   <si>
-    <t>В работе. Договоры проходят процедуру согласования в ПС</t>
-  </si>
-  <si>
     <t>выполнено. Согласован В.Ксенофонтовым 13.10.26. Ожидается согласование Н.Луканихиной 20.10.26</t>
   </si>
   <si>
@@ -253,12 +247,6 @@
   </si>
   <si>
     <t>Установка звукового и светового оборудования в Лофте</t>
-  </si>
-  <si>
-    <t>Выполнено. 23.10.26 Ожидается поставка бочек и гирлянды</t>
-  </si>
-  <si>
-    <t>20.10.26 будет тест экрана</t>
   </si>
 </sst>
 </file>
@@ -456,6 +444,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -464,9 +455,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -697,13 +685,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" ht="24" customHeight="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="24"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="25"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="10"/>
@@ -733,7 +721,7 @@
       <c r="A5" s="10">
         <v>1</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="C5" s="9">
@@ -750,7 +738,7 @@
       <c r="A6" s="10">
         <v>2</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="22" t="s">
         <v>28</v>
       </c>
       <c r="C6" s="9">
@@ -767,7 +755,7 @@
       <c r="A7" s="10">
         <v>3</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="22" t="s">
         <v>29</v>
       </c>
       <c r="C7" s="9">
@@ -784,7 +772,7 @@
       <c r="A8" s="10">
         <v>4</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="22" t="s">
         <v>30</v>
       </c>
       <c r="C8" s="9">
@@ -801,7 +789,7 @@
       <c r="A9" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="22" t="s">
         <v>62</v>
       </c>
       <c r="C9" s="9">
@@ -818,7 +806,7 @@
       <c r="A10" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="22" t="s">
         <v>61</v>
       </c>
       <c r="C10" s="9">
@@ -835,7 +823,7 @@
       <c r="A11" s="10">
         <v>5</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="22" t="s">
         <v>31</v>
       </c>
       <c r="C11" s="9">
@@ -845,14 +833,14 @@
         <v>46280</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="51.5" customHeight="1">
       <c r="A12" s="10">
         <v>6</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="22" t="s">
         <v>32</v>
       </c>
       <c r="C12" s="9">
@@ -862,14 +850,14 @@
         <v>46280</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="45.5" customHeight="1">
       <c r="A13" s="10">
         <v>7</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="22" t="s">
         <v>63</v>
       </c>
       <c r="C13" s="9">
@@ -886,7 +874,7 @@
       <c r="A14" s="10">
         <v>8</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="22" t="s">
         <v>22</v>
       </c>
       <c r="C14" s="20">
@@ -896,7 +884,7 @@
         <v>46290</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="20" customHeight="1">
@@ -954,7 +942,7 @@
       <c r="A18" s="10">
         <v>9</v>
       </c>
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="22" t="s">
         <v>16</v>
       </c>
       <c r="C18" s="19">
@@ -964,7 +952,9 @@
       <c r="D18" s="19">
         <v>46320</v>
       </c>
-      <c r="E18" s="1"/>
+      <c r="E18" s="18" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="19" spans="1:5" ht="20" customHeight="1">
       <c r="A19" s="10" t="s">
@@ -1030,7 +1020,9 @@
       <c r="D22" s="19">
         <v>46318</v>
       </c>
-      <c r="E22" s="1"/>
+      <c r="E22" s="18" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="23" spans="1:5" ht="20" customHeight="1">
       <c r="A23" s="10" t="s">
@@ -1088,7 +1080,7 @@
         <v>48</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C26" s="6">
         <v>46286</v>
@@ -1097,7 +1089,7 @@
         <v>46307</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>68</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="30" customHeight="1">
@@ -1105,7 +1097,7 @@
         <v>49</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C27" s="6">
         <v>46296</v>
@@ -1114,7 +1106,7 @@
         <v>10</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>72</v>
+        <v>38</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="36" customHeight="1">
@@ -1156,7 +1148,7 @@
         <v>52</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C30" s="6">
         <v>46315</v>
@@ -1164,8 +1156,8 @@
       <c r="D30" s="6">
         <v>46317</v>
       </c>
-      <c r="E30" s="5" t="s">
-        <v>73</v>
+      <c r="E30" s="18" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="36" customHeight="1">
@@ -1181,8 +1173,8 @@
       <c r="D31" s="6">
         <v>46317</v>
       </c>
-      <c r="E31" s="5" t="s">
-        <v>64</v>
+      <c r="E31" s="18" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="36" customHeight="1">
@@ -1198,7 +1190,9 @@
       <c r="D32" s="6">
         <v>46318</v>
       </c>
-      <c r="E32" s="5"/>
+      <c r="E32" s="18" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="33" spans="1:5" ht="36" customHeight="1">
       <c r="A33" s="4" t="s">
@@ -1213,7 +1207,9 @@
       <c r="D33" s="6">
         <v>46318</v>
       </c>
-      <c r="E33" s="5"/>
+      <c r="E33" s="18" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="34" spans="1:5" ht="36" customHeight="1">
       <c r="A34" s="4" t="s">
@@ -1228,13 +1224,15 @@
       <c r="D34" s="6">
         <v>46318</v>
       </c>
-      <c r="E34" s="5"/>
+      <c r="E34" s="18" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="35" spans="1:5" ht="24.5" customHeight="1">
       <c r="A35" s="12">
         <v>11</v>
       </c>
-      <c r="B35" s="25" t="s">
+      <c r="B35" s="22" t="s">
         <v>20</v>
       </c>
       <c r="C35" s="19">
@@ -1243,13 +1241,15 @@
       <c r="D35" s="19">
         <v>46318</v>
       </c>
-      <c r="E35" s="5"/>
+      <c r="E35" s="18" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="36" spans="1:5" ht="25.5" customHeight="1">
       <c r="A36" s="12">
         <v>12</v>
       </c>
-      <c r="B36" s="25" t="s">
+      <c r="B36" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C36" s="19">
@@ -1258,7 +1258,9 @@
       <c r="D36" s="19">
         <v>46320</v>
       </c>
-      <c r="E36" s="5"/>
+      <c r="E36" s="18" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="37" spans="1:5" ht="36" customHeight="1">
       <c r="B37" s="17"/>

</xml_diff>